<commit_message>
move neighbor reveal to option
</commit_message>
<xml_diff>
--- a/docs/graph-plus-ui-interaction-matrix.xlsx
+++ b/docs/graph-plus-ui-interaction-matrix.xlsx
@@ -2,20 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Index" sheetId="1" r:id="R65e8b62d37c54fd1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Definitions" sheetId="2" r:id="R342d775b3c2148b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Desktop Pointer" sheetId="3" r:id="R05a756a7417d4ed3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Desktop Trackpad" sheetId="4" r:id="R027d48a9707e463a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keyboard" sheetId="5" r:id="Rdc9876a903ef4fda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mobile Touch" sheetId="6" r:id="Rc86dc48e83144aba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mobile Two-Finger" sheetId="7" r:id="R13fdf6124aea4caa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stylus" sheetId="8" r:id="R29aca89dcef54fd2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Centering" sheetId="9" r:id="R18a22b517019465c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Node Context Menu" sheetId="10" r:id="R1e2f4085e075453d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Settings UI" sheetId="11" r:id="Ra773dfd67c834a58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Settings Controls" sheetId="12" r:id="R5714d99ffe8c4182"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Note Preview" sheetId="13" r:id="Rd724abbf05cd4abd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Decisions" sheetId="14" r:id="R7a42803be5e24a73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Index" sheetId="1" r:id="Rc4d5776214704208"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Definitions" sheetId="2" r:id="Rd70a2c68d87a4a4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Desktop Pointer" sheetId="3" r:id="R6682b37d56a24093"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Desktop Trackpad" sheetId="4" r:id="R63a0114a9559425e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keyboard" sheetId="5" r:id="Ra8a20845ebda481e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mobile Touch" sheetId="6" r:id="Rae6ff21234a440a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mobile Two-Finger" sheetId="7" r:id="R111c622533fb4402"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stylus" sheetId="8" r:id="Rf01fb911478b46b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Centering" sheetId="9" r:id="R9336df5a65df425f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Node Context Menu" sheetId="10" r:id="R482dfe65825b48e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Settings UI" sheetId="11" r:id="Rf955a9bfb2124656"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Settings Controls" sheetId="12" r:id="Rf64454b413fd4f15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Note Preview" sheetId="13" r:id="R30677a2b9ae04cd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Decisions" sheetId="14" r:id="R19cef98dad454bff"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26,7 +26,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="6">
+  <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -60,8 +60,18 @@
       <x:color rgb="FF216E39"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF8A6D1F"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF2E7D32"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="31">
+  <x:fills count="33">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -213,6 +223,16 @@
         <x:fgColor rgb="FFE8F3EC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="6">
     <x:border/>
@@ -260,7 +280,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="75">
+  <x:cellXfs count="79">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -470,6 +490,18 @@
     <x:xf numFmtId="0" fontId="5" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -2278,18 +2310,18 @@
         <x:color rgb="FF7A5200"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFFF4D6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF216E39"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF216E39"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
           <x:bgColor rgb="FFE8F3EC"/>
         </x:patternFill>
       </x:fill>
@@ -2300,7 +2332,7 @@
         <x:color rgb="FF9C2F23"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFBE9E7"/>
         </x:patternFill>
       </x:fill>
@@ -2310,18 +2342,18 @@
         <x:color rgb="FF7A5200"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFFF4D6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF216E39"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF216E39"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
           <x:bgColor rgb="FFE8F3EC"/>
         </x:patternFill>
       </x:fill>
@@ -2332,7 +2364,7 @@
         <x:color rgb="FF9C2F23"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFBE9E7"/>
         </x:patternFill>
       </x:fill>
@@ -2342,18 +2374,18 @@
         <x:color rgb="FF7A5200"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFFF4D6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF216E39"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF216E39"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
           <x:bgColor rgb="FFE8F3EC"/>
         </x:patternFill>
       </x:fill>
@@ -2364,7 +2396,7 @@
         <x:color rgb="FF9C2F23"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFBE9E7"/>
         </x:patternFill>
       </x:fill>
@@ -2374,18 +2406,18 @@
         <x:color rgb="FF7A5200"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFFF4D6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF216E39"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF216E39"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
           <x:bgColor rgb="FFE8F3EC"/>
         </x:patternFill>
       </x:fill>
@@ -2396,7 +2428,7 @@
         <x:color rgb="FF9C2F23"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFBE9E7"/>
         </x:patternFill>
       </x:fill>
@@ -2406,18 +2438,18 @@
         <x:color rgb="FF7A5200"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFFF4D6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF216E39"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF216E39"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
           <x:bgColor rgb="FFE8F3EC"/>
         </x:patternFill>
       </x:fill>
@@ -2428,7 +2460,7 @@
         <x:color rgb="FF9C2F23"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFBE9E7"/>
         </x:patternFill>
       </x:fill>
@@ -2719,10 +2751,10 @@
         <x:v>Keyboard</x:v>
       </x:c>
       <x:c r="B9" s="18" t="str">
-        <x:v>This matrix applies on desktop and on mobile when a hardware keyboard is present.</x:v>
+        <x:v>This matrix applies on desktop and on mobile when a hardware keyboard is present. Ctrl edits selection; Option temporarily reveals selection neighbors and connecting links.</x:v>
       </x:c>
       <x:c r="C9" s="18" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="D9" s="21" t="str">
         <x:v>Open</x:v>
@@ -2857,7 +2889,7 @@
         <x:v>Resolved decisions from UI contract review.</x:v>
       </x:c>
       <x:c r="C18" s="19" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="D18" s="20" t="str">
         <x:v>Approved</x:v>
@@ -3734,12 +3766,12 @@
         <x:v>Conditional Center + Fit</x:v>
       </x:c>
       <x:c r="C12" s="19" t="str">
-        <x:v>While Ctrl is held, undim direct neighbors of the current selection and update that reveal as selection changes. On release, restore normal dimming. Center + Fit only after an initial selection that began empty; otherwise no camera change.</x:v>
+        <x:v>Center + Fit only after an initial selection that began empty; otherwise no camera change.</x:v>
       </x:c>
       <x:c r="D12" s="20" t="str">
         <x:v>Approved</x:v>
       </x:c>
-      <x:c r="E12" s="19" t="str"/>
+      <x:c r="E12" s="19"/>
     </x:row>
     <x:row r="13" ht="43" customHeight="1">
       <x:c r="A13" s="18" t="str">
@@ -3755,6 +3787,21 @@
         <x:v>Approved</x:v>
       </x:c>
       <x:c r="E13" s="18" t="str"/>
+    </x:row>
+    <x:row r="14" ht="60" customHeight="1">
+      <x:c r="A14" s="43" t="str">
+        <x:v>Option neighbor reveal</x:v>
+      </x:c>
+      <x:c r="B14" s="43" t="str">
+        <x:v>Transient selection presentation</x:v>
+      </x:c>
+      <x:c r="C14" s="43" t="str">
+        <x:v>While Option is held, undim direct neighbors of the current selection and the links connecting them to the selection. Update the reveal as selection changes. On release, restore normal dimming without changing selection, focus, or camera.</x:v>
+      </x:c>
+      <x:c r="D14" s="78" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+      <x:c r="E14" s="43"/>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="D6:D13">
@@ -3762,9 +3809,12 @@
     <x:cfRule type="containsText" dxfId="58" priority="2" operator="containsText" text="Change"/>
     <x:cfRule type="containsText" dxfId="59" priority="3" operator="containsText" text="Open"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="1">
+  <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="D6:D13">
       <x:formula1>"Open,Approved,Change"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="D14">
+      <x:formula1>"Open,Approved,Needs changes"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4262,7 +4312,7 @@
         <x:v>Same</x:v>
       </x:c>
       <x:c r="E14" s="19" t="str">
-        <x:v>Update selection and centroid without moving focus; while Ctrl is held, undim direct neighbors of the current selection</x:v>
+        <x:v>Update selection and centroid without moving focus</x:v>
       </x:c>
       <x:c r="F14" s="19" t="str">
         <x:v>Confirmed requirement</x:v>
@@ -4286,7 +4336,7 @@
         <x:v>Same</x:v>
       </x:c>
       <x:c r="E15" s="18" t="str">
-        <x:v>Update selection and centroid without moving focus; while Ctrl is held, undim direct neighbors of the current selection</x:v>
+        <x:v>Update selection and centroid without moving focus</x:v>
       </x:c>
       <x:c r="F15" s="18" t="str">
         <x:v>Confirmed requirement</x:v>
@@ -4310,7 +4360,7 @@
         <x:v>Same</x:v>
       </x:c>
       <x:c r="E16" s="19" t="str">
-        <x:v>Keep resulting selection; set focus to its centroid; restore normal selection dimming</x:v>
+        <x:v>Keep resulting selection; set focus to its centroid</x:v>
       </x:c>
       <x:c r="F16" s="19" t="str">
         <x:v>Confirmed requirement</x:v>
@@ -4334,7 +4384,7 @@
         <x:v>Same</x:v>
       </x:c>
       <x:c r="E17" s="18" t="str">
-        <x:v>Keep additions and removals; keep the existing focus point; restore normal selection dimming</x:v>
+        <x:v>Keep additions and removals; keep the existing focus point</x:v>
       </x:c>
       <x:c r="F17" s="18" t="str">
         <x:v>Confirmed requirement</x:v>
@@ -5034,13 +5084,13 @@
         <x:v>Hold Ctrl</x:v>
       </x:c>
       <x:c r="B13" s="18" t="str">
-        <x:v>Undim direct neighbors of the current selection</x:v>
+        <x:v>Enable additive or removal selection</x:v>
       </x:c>
       <x:c r="C13" s="18" t="str">
         <x:v>Same</x:v>
       </x:c>
       <x:c r="D13" s="18" t="str">
-        <x:v>While held, reveal direct neighbors and enable additive or removal selection; update the revealed neighborhood as selection changes</x:v>
+        <x:v>Do not change presentation or camera while held; additions and removals recalculate the centroid without moving focus</x:v>
       </x:c>
       <x:c r="E13" s="18" t="str">
         <x:v>Confirmed requirement</x:v>
@@ -5052,16 +5102,16 @@
     </x:row>
     <x:row r="14" ht="43" customHeight="1">
       <x:c r="A14" s="19" t="str">
-        <x:v>Release Ctrl after editing an existing selection</x:v>
+        <x:v>Hold Option</x:v>
       </x:c>
       <x:c r="B14" s="19" t="str">
-        <x:v>No camera change</x:v>
+        <x:v>Undim direct neighbors of the current selection and the links connecting them to the selection</x:v>
       </x:c>
       <x:c r="C14" s="19" t="str">
-        <x:v>No camera change</x:v>
+        <x:v>Same</x:v>
       </x:c>
       <x:c r="D14" s="19" t="str">
-        <x:v>Keep additions and removals; recalculate the centroid without moving focus; restore normal selection dimming</x:v>
+        <x:v>Do not mutate selection, focus, or camera; update the reveal as selection changes; release restores normal dimming</x:v>
       </x:c>
       <x:c r="E14" s="19" t="str">
         <x:v>Confirmed requirement</x:v>
@@ -5073,16 +5123,16 @@
     </x:row>
     <x:row r="15" ht="43" customHeight="1">
       <x:c r="A15" s="18" t="str">
-        <x:v>Release Ctrl after initial selection</x:v>
+        <x:v>Release Ctrl after editing an existing selection</x:v>
       </x:c>
       <x:c r="B15" s="18" t="str">
-        <x:v>Center + Fit</x:v>
+        <x:v>No camera change</x:v>
       </x:c>
       <x:c r="C15" s="18" t="str">
-        <x:v>Center + Fit</x:v>
+        <x:v>No camera change</x:v>
       </x:c>
       <x:c r="D15" s="18" t="str">
-        <x:v>Keep resulting selection; set focus to its centroid; restore normal selection dimming</x:v>
+        <x:v>Keep additions and removals; recalculate the centroid without moving focus</x:v>
       </x:c>
       <x:c r="E15" s="18" t="str">
         <x:v>Confirmed requirement</x:v>
@@ -5094,37 +5144,37 @@
     </x:row>
     <x:row r="16" ht="43" customHeight="1">
       <x:c r="A16" s="19" t="str">
-        <x:v>Tab on graph or background</x:v>
+        <x:v>Release Ctrl after initial selection</x:v>
       </x:c>
       <x:c r="B16" s="19" t="str">
-        <x:v>Toggle Quick Settings</x:v>
+        <x:v>Center + Fit</x:v>
       </x:c>
       <x:c r="C16" s="19" t="str">
-        <x:v>Same</x:v>
+        <x:v>Center + Fit</x:v>
       </x:c>
       <x:c r="D16" s="19" t="str">
-        <x:v>Disabled while typing in a control</x:v>
+        <x:v>Keep resulting selection; set focus to its centroid</x:v>
       </x:c>
       <x:c r="E16" s="19" t="str">
-        <x:v>Current</x:v>
+        <x:v>Confirmed requirement</x:v>
       </x:c>
       <x:c r="F16" s="20" t="str">
-        <x:v>Open</x:v>
-      </x:c>
-      <x:c r="G16" s="19" t="str"/>
+        <x:v>Approved</x:v>
+      </x:c>
+      <x:c r="G16" s="19"/>
     </x:row>
     <x:row r="17" ht="43" customHeight="1">
       <x:c r="A17" s="18" t="str">
-        <x:v>Shift + Tab</x:v>
+        <x:v>Tab on graph or background</x:v>
       </x:c>
       <x:c r="B17" s="18" t="str">
-        <x:v>Normal reverse focus navigation</x:v>
+        <x:v>Toggle Quick Settings</x:v>
       </x:c>
       <x:c r="C17" s="18" t="str">
         <x:v>Same</x:v>
       </x:c>
       <x:c r="D17" s="18" t="str">
-        <x:v>Do not toggle panel</x:v>
+        <x:v>Disabled while typing in a control</x:v>
       </x:c>
       <x:c r="E17" s="18" t="str">
         <x:v>Current</x:v>
@@ -5132,20 +5182,20 @@
       <x:c r="F17" s="21" t="str">
         <x:v>Open</x:v>
       </x:c>
-      <x:c r="G17" s="18" t="str"/>
+      <x:c r="G17" s="18"/>
     </x:row>
     <x:row r="18" ht="43" customHeight="1">
       <x:c r="A18" s="19" t="str">
-        <x:v>0 or F</x:v>
+        <x:v>Shift + Tab</x:v>
       </x:c>
       <x:c r="B18" s="19" t="str">
-        <x:v>No graph action</x:v>
+        <x:v>Normal reverse focus navigation</x:v>
       </x:c>
       <x:c r="C18" s="19" t="str">
-        <x:v>No graph action</x:v>
+        <x:v>Same</x:v>
       </x:c>
       <x:c r="D18" s="19" t="str">
-        <x:v>None</x:v>
+        <x:v>Do not toggle panel</x:v>
       </x:c>
       <x:c r="E18" s="19" t="str">
         <x:v>Current</x:v>
@@ -5153,7 +5203,28 @@
       <x:c r="F18" s="20" t="str">
         <x:v>Open</x:v>
       </x:c>
-      <x:c r="G18" s="19" t="str"/>
+      <x:c r="G18" s="19"/>
+    </x:row>
+    <x:row r="19" ht="43" customHeight="1">
+      <x:c r="A19" s="43" t="str">
+        <x:v>0 or F</x:v>
+      </x:c>
+      <x:c r="B19" s="43" t="str">
+        <x:v>No graph action</x:v>
+      </x:c>
+      <x:c r="C19" s="43" t="str">
+        <x:v>No graph action</x:v>
+      </x:c>
+      <x:c r="D19" s="43" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="E19" s="43" t="str">
+        <x:v>Current</x:v>
+      </x:c>
+      <x:c r="F19" s="76" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="G19" s="43"/>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="F6:F18">
@@ -5165,9 +5236,12 @@
     <x:cfRule type="containsText" dxfId="19" priority="4" operator="containsText" text="Confirmed"/>
     <x:cfRule type="containsText" dxfId="20" priority="5" operator="containsText" text="Verify"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="1">
+  <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="F6:F18">
       <x:formula1>"Open,Approved,Change"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="F19">
+      <x:formula1>"Open,Approved,Needs changes"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
align tag and modifier interactions
</commit_message>
<xml_diff>
--- a/docs/graph-plus-ui-interaction-matrix.xlsx
+++ b/docs/graph-plus-ui-interaction-matrix.xlsx
@@ -2,20 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Index" sheetId="1" r:id="Rc4d5776214704208"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Definitions" sheetId="2" r:id="Rd70a2c68d87a4a4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Desktop Pointer" sheetId="3" r:id="R6682b37d56a24093"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Desktop Trackpad" sheetId="4" r:id="R63a0114a9559425e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keyboard" sheetId="5" r:id="Ra8a20845ebda481e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mobile Touch" sheetId="6" r:id="Rae6ff21234a440a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mobile Two-Finger" sheetId="7" r:id="R111c622533fb4402"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stylus" sheetId="8" r:id="Rf01fb911478b46b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Centering" sheetId="9" r:id="R9336df5a65df425f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Node Context Menu" sheetId="10" r:id="R482dfe65825b48e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Settings UI" sheetId="11" r:id="Rf955a9bfb2124656"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Settings Controls" sheetId="12" r:id="Rf64454b413fd4f15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Note Preview" sheetId="13" r:id="R30677a2b9ae04cd4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Decisions" sheetId="14" r:id="R19cef98dad454bff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Index" sheetId="1" r:id="Ra3036747682d4622"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Definitions" sheetId="2" r:id="R2817250ff5bb47f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Desktop Pointer" sheetId="3" r:id="R1d2fc27db3c0483c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Desktop Trackpad" sheetId="4" r:id="R39d6984029164fe8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keyboard" sheetId="5" r:id="Rf9c2bea826fc4e5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mobile Touch" sheetId="6" r:id="R99eaa93ef4cd4097"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mobile Two-Finger" sheetId="7" r:id="R74bef573dbd041b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stylus" sheetId="8" r:id="R5473d00fb3ce4f87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Centering" sheetId="9" r:id="R3bb2c2cd78c94391"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Node Context Menu" sheetId="10" r:id="R21b758f890064144"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Settings UI" sheetId="11" r:id="Ra98b58b2463d4b22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Settings Controls" sheetId="12" r:id="R4c31caa2f86c431d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Note Preview" sheetId="13" r:id="Rddec7262cf5e482d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Decisions" sheetId="14" r:id="Rb129716c536b49aa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -71,7 +71,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="33">
+  <x:fills count="34">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -233,6 +233,11 @@
         <x:fgColor rgb="FFE2F0D9"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="6">
     <x:border/>
@@ -280,7 +285,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="79">
+  <x:cellXfs count="81">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -500,6 +505,12 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2739,7 +2750,7 @@
         <x:v>A browser usually reports physical mouse-wheel and two-finger trackpad scroll through the same wheel event path.</x:v>
       </x:c>
       <x:c r="C8" s="19" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="D8" s="20" t="str">
         <x:v>Open</x:v>
@@ -2889,7 +2900,7 @@
         <x:v>Resolved decisions from UI contract review.</x:v>
       </x:c>
       <x:c r="C18" s="19" t="n">
-        <x:v>9</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D18" s="20" t="str">
         <x:v>Approved</x:v>
@@ -3790,18 +3801,48 @@
     </x:row>
     <x:row r="14" ht="60" customHeight="1">
       <x:c r="A14" s="43" t="str">
-        <x:v>Option neighbor reveal</x:v>
+        <x:v>Option neighbor highlight</x:v>
       </x:c>
       <x:c r="B14" s="43" t="str">
-        <x:v>Transient selection presentation</x:v>
+        <x:v>Transient hover-equivalent presentation</x:v>
       </x:c>
       <x:c r="C14" s="43" t="str">
-        <x:v>While Option is held, undim direct neighbors of the current selection and the links connecting them to the selection. Update the reveal as selection changes. On release, restore normal dimming without changing selection, focus, or camera.</x:v>
+        <x:v>While Option is held, highlight direct neighbors of the current selection and the links connecting them to the selection using the same treatment as hovering the selected node. Update the highlight as selection changes. On release, restore normal presentation without changing selection, focus, or camera.</x:v>
       </x:c>
       <x:c r="D14" s="78" t="str">
         <x:v>Approved</x:v>
       </x:c>
       <x:c r="E14" s="43"/>
+    </x:row>
+    <x:row r="15" ht="60" customHeight="1">
+      <x:c r="A15" s="43" t="str">
+        <x:v>Tag node selection</x:v>
+      </x:c>
+      <x:c r="B15" s="43" t="str">
+        <x:v>Same as ordinary node selection</x:v>
+      </x:c>
+      <x:c r="C15" s="43" t="str">
+        <x:v>Clicking a tag selects only that tag. Region members remain unselected and do not receive selected-label presentation.</x:v>
+      </x:c>
+      <x:c r="D15" s="80" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+      <x:c r="E15" s="43"/>
+    </x:row>
+    <x:row r="16" ht="60" customHeight="1">
+      <x:c r="A16" s="43" t="str">
+        <x:v>Cmd-scroll</x:v>
+      </x:c>
+      <x:c r="B16" s="43" t="str">
+        <x:v>Ordinary wheel navigation</x:v>
+      </x:c>
+      <x:c r="C16" s="43" t="str">
+        <x:v>Cmd does not enable zoom. Cmd-scroll follows the same 2D and 3D navigation behavior as unmodified wheel input.</x:v>
+      </x:c>
+      <x:c r="D16" s="80" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+      <x:c r="E16" s="43"/>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="D6:D13">
@@ -3809,11 +3850,17 @@
     <x:cfRule type="containsText" dxfId="58" priority="2" operator="containsText" text="Change"/>
     <x:cfRule type="containsText" dxfId="59" priority="3" operator="containsText" text="Open"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="2">
+  <x:dataValidations count="4">
     <x:dataValidation type="list" sqref="D6:D13">
       <x:formula1>"Open,Approved,Change"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="D14">
+      <x:formula1>"Open,Approved,Needs changes"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="D15">
+      <x:formula1>"Open,Approved,Needs changes"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="D16">
       <x:formula1>"Open,Approved,Needs changes"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -4231,16 +4278,16 @@
         <x:v>Primary click</x:v>
       </x:c>
       <x:c r="B11" s="18" t="str">
-        <x:v>Node, no existing selection</x:v>
+        <x:v>Node, including tag, with no existing selection</x:v>
       </x:c>
       <x:c r="C11" s="18" t="str">
-        <x:v>On release, select node; then Center + Fit selection</x:v>
+        <x:v>On release, select only the clicked node; then Center + Fit selection</x:v>
       </x:c>
       <x:c r="D11" s="18" t="str">
         <x:v>Same</x:v>
       </x:c>
       <x:c r="E11" s="18" t="str">
-        <x:v>Begin selection; set focus point to the calculated selection centroid</x:v>
+        <x:v>Begin selection with only the clicked node; set focus point to the calculated selection centroid</x:v>
       </x:c>
       <x:c r="F11" s="18" t="str">
         <x:v>Confirmed requirement</x:v>
@@ -4255,16 +4302,16 @@
         <x:v>Primary click</x:v>
       </x:c>
       <x:c r="B12" s="19" t="str">
-        <x:v>Node, existing selection</x:v>
+        <x:v>Node, including tag, with an existing selection</x:v>
       </x:c>
       <x:c r="C12" s="19" t="str">
-        <x:v>On release, add node and shortest-path bridge; no camera change</x:v>
+        <x:v>On release, add the clicked node and shortest-path bridge; no camera change</x:v>
       </x:c>
       <x:c r="D12" s="19" t="str">
         <x:v>Same</x:v>
       </x:c>
       <x:c r="E12" s="19" t="str">
-        <x:v>Accumulate selection and recalculate its centroid; keep the existing focus point</x:v>
+        <x:v>Accumulate the clicked node and bridge; recalculate the centroid; keep the existing focus point</x:v>
       </x:c>
       <x:c r="F12" s="19" t="str">
         <x:v>Confirmed requirement</x:v>
@@ -4864,6 +4911,27 @@
       </x:c>
       <x:c r="G13" s="18" t="str"/>
     </x:row>
+    <x:row r="14" ht="43" customHeight="1">
+      <x:c r="A14" s="43" t="str">
+        <x:v>Cmd + two-finger scroll or wheel</x:v>
+      </x:c>
+      <x:c r="B14" s="43" t="str">
+        <x:v>Any</x:v>
+      </x:c>
+      <x:c r="C14" s="43" t="str">
+        <x:v>Same as unmodified</x:v>
+      </x:c>
+      <x:c r="D14" s="43" t="str">
+        <x:v>Same as unmodified</x:v>
+      </x:c>
+      <x:c r="E14" s="43" t="str">
+        <x:v>Cmd does not enable zoom</x:v>
+      </x:c>
+      <x:c r="F14" s="80" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+      <x:c r="G14" s="43"/>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="F6:F13">
     <x:cfRule type="containsText" dxfId="11" priority="1" operator="containsText" text="Approved"/>
@@ -4874,9 +4942,12 @@
     <x:cfRule type="containsText" dxfId="14" priority="4" operator="containsText" text="Confirmed"/>
     <x:cfRule type="containsText" dxfId="15" priority="5" operator="containsText" text="Verify"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="1">
+  <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="F6:F13">
       <x:formula1>"Open,Approved,Change"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="F14">
+      <x:formula1>"Open,Approved,Needs changes"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5105,13 +5176,13 @@
         <x:v>Hold Option</x:v>
       </x:c>
       <x:c r="B14" s="19" t="str">
-        <x:v>Undim direct neighbors of the current selection and the links connecting them to the selection</x:v>
+        <x:v>Highlight direct neighbors of the current selection and the links connecting them to the selection</x:v>
       </x:c>
       <x:c r="C14" s="19" t="str">
         <x:v>Same</x:v>
       </x:c>
       <x:c r="D14" s="19" t="str">
-        <x:v>Do not mutate selection, focus, or camera; update the reveal as selection changes; release restores normal dimming</x:v>
+        <x:v>Use the same highlight treatment as hovering the selected node; do not mutate selection, focus, or camera; release restores normal selection presentation</x:v>
       </x:c>
       <x:c r="E14" s="19" t="str">
         <x:v>Confirmed requirement</x:v>

</xml_diff>

<commit_message>
document mobile background rotate
</commit_message>
<xml_diff>
--- a/docs/graph-plus-ui-interaction-matrix.xlsx
+++ b/docs/graph-plus-ui-interaction-matrix.xlsx
@@ -2,20 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Index" sheetId="1" r:id="Ra3036747682d4622"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Definitions" sheetId="2" r:id="R2817250ff5bb47f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Desktop Pointer" sheetId="3" r:id="R1d2fc27db3c0483c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Desktop Trackpad" sheetId="4" r:id="R39d6984029164fe8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keyboard" sheetId="5" r:id="Rf9c2bea826fc4e5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mobile Touch" sheetId="6" r:id="R99eaa93ef4cd4097"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mobile Two-Finger" sheetId="7" r:id="R74bef573dbd041b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stylus" sheetId="8" r:id="R5473d00fb3ce4f87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Centering" sheetId="9" r:id="R3bb2c2cd78c94391"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Node Context Menu" sheetId="10" r:id="R21b758f890064144"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Settings UI" sheetId="11" r:id="Ra98b58b2463d4b22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Settings Controls" sheetId="12" r:id="R4c31caa2f86c431d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Note Preview" sheetId="13" r:id="Rddec7262cf5e482d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Decisions" sheetId="14" r:id="Rb129716c536b49aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Index" sheetId="1" r:id="R67eaa48484b342ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Definitions" sheetId="2" r:id="R1b9068ba29024758"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Desktop Pointer" sheetId="3" r:id="R80827e993d564b9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Desktop Trackpad" sheetId="4" r:id="Rcff5a4f6383c491a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keyboard" sheetId="5" r:id="R80cc330924df4b46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mobile Touch" sheetId="6" r:id="R20dcd0a9aed14a9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mobile Two-Finger" sheetId="7" r:id="Rb2d5c2b1756049f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stylus" sheetId="8" r:id="R92f0485f2e664292"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Centering" sheetId="9" r:id="R7922007b4a4e4adb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Node Context Menu" sheetId="10" r:id="Re268440acfbc49a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Settings UI" sheetId="11" r:id="R60e199a014e0472e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Settings Controls" sheetId="12" r:id="Rf3c03185b98f41ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Note Preview" sheetId="13" r:id="R3726414233ec42f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Decisions" sheetId="14" r:id="Ra3dc5d7ab4c34f32"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5343,7 +5343,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="str">
-        <x:v>Two-finger behavior is defined separately. One-finger background behavior remains open for review.</x:v>
+        <x:v>Two-finger behavior is defined separately. One-finger background drag pans in 2D and rotates the camera in 3D.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
@@ -5455,13 +5455,13 @@
         <x:v>Pan</x:v>
       </x:c>
       <x:c r="D9" s="18" t="str">
-        <x:v>Currently pans</x:v>
+        <x:v>Rotate camera</x:v>
       </x:c>
       <x:c r="E9" s="18" t="str">
-        <x:v>Preserve selection state; pan translates the stored focus point</x:v>
+        <x:v>No selection change; 2D pan translates the stored focus point and 3D rotate uses it</x:v>
       </x:c>
       <x:c r="F9" s="18" t="str">
-        <x:v>Verify intended 3D behavior</x:v>
+        <x:v>Confirmed requirement</x:v>
       </x:c>
       <x:c r="G9" s="21" t="str">
         <x:v>Approved</x:v>

</xml_diff>

<commit_message>
refactor(graph-engine): split animus and anima
</commit_message>
<xml_diff>
--- a/docs/graph-plus-ui-interaction-matrix.xlsx
+++ b/docs/graph-plus-ui-interaction-matrix.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Index" sheetId="1" r:id="Rcfd0f9b4156c4995"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Definitions" sheetId="2" r:id="Rdd49707a76cb4b93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Desktop Pointer" sheetId="3" r:id="Rdcf6c81473214bf1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Desktop Trackpad" sheetId="4" r:id="R11c0f3b7a157433b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keyboard" sheetId="5" r:id="Ra2c6f2646cee46c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mobile Touch" sheetId="6" r:id="R54a5b1f2059040d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mobile Two-Finger" sheetId="7" r:id="R5e7a25f455b2438d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stylus" sheetId="8" r:id="R4324de4c009c4e16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Centering" sheetId="9" r:id="R3cf89ac732934a4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Node Context Menu" sheetId="10" r:id="Rf89cde0c37f74a2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Settings UI" sheetId="11" r:id="R49081ccca45e4558"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Settings Controls" sheetId="12" r:id="R322368a5ede9427b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Note Preview" sheetId="13" r:id="Rcaa7840dae554503"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Decisions" sheetId="14" r:id="R829c9ad958fc431d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Policies" sheetId="15" r:id="Rf0ccd3ada4664672"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Transitions" sheetId="16" r:id="R0426697231f84912"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Focus Rendering" sheetId="17" r:id="R9623b98e3cb14706"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Index" sheetId="1" r:id="R8cc5b61620864eea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Definitions" sheetId="2" r:id="Rb85033a6d181416e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Desktop Pointer" sheetId="3" r:id="R07cd7d55ef7a476e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Desktop Trackpad" sheetId="4" r:id="R3c19a54f1dbc4108"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keyboard" sheetId="5" r:id="R7ce3b2f2a906428c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mobile Touch" sheetId="6" r:id="Re7ac96b293ed4fca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mobile Two-Finger" sheetId="7" r:id="Rd2463b5dcd0d4988"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stylus" sheetId="8" r:id="Ra9e0cce182d5419d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Centering" sheetId="9" r:id="R818365b1f8fc4837"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Node Context Menu" sheetId="10" r:id="Reefb1635313048b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Settings UI" sheetId="11" r:id="R70af8ee51a244a2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Settings Controls" sheetId="12" r:id="R13f8e582173049af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Note Preview" sheetId="13" r:id="R7553edd5b3774a5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Decisions" sheetId="14" r:id="R8cf13a0cd7f84ee0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Policies" sheetId="15" r:id="Rc470dda50a7945f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Transitions" sheetId="16" r:id="R675a458e26314751"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Focus Rendering" sheetId="17" r:id="R2f741878f89b4729"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3137,7 +3137,7 @@
         <x:v>All state-changing stationary activations</x:v>
       </x:c>
       <x:c r="C8" s="101" t="n">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D8" s="103" t="str">
         <x:v>Approved</x:v>
@@ -3360,7 +3360,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd118e2cbf286437c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfea1b0e8c1b145f4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3519,7 +3519,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4433e7ef8205426d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb502d435a5244c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4320,7 +4320,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a37b8e369f548e9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58a39c9bc09b4f29"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4419,7 +4419,7 @@
         <x:v>Whole graph</x:v>
       </x:c>
       <x:c r="F6" s="101" t="str">
-        <x:v>Whole graph</x:v>
+        <x:v>Whole graph; context normal</x:v>
       </x:c>
       <x:c r="G6" s="101" t="str">
         <x:v>Pan</x:v>
@@ -4445,7 +4445,7 @@
         <x:v>Selection</x:v>
       </x:c>
       <x:c r="F7" s="105" t="str">
-        <x:v>Graph with selection emphasis</x:v>
+        <x:v>Whole graph; selection highlighted, context dimmed</x:v>
       </x:c>
       <x:c r="G7" s="105" t="str">
         <x:v>Pan</x:v>
@@ -4471,7 +4471,7 @@
         <x:v>Focused node + immediate neighbors</x:v>
       </x:c>
       <x:c r="F8" s="101" t="str">
-        <x:v>Focused local view</x:v>
+        <x:v>Focused local view; local highlighted, other context hidden</x:v>
       </x:c>
       <x:c r="G8" s="101" t="str">
         <x:v>Elastic pan</x:v>
@@ -4483,7 +4483,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42ff5286e68945e9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b5965d5a41445ae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4788,10 +4788,33 @@
         <x:v>No implicit fit</x:v>
       </x:c>
     </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>Focus</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>Release Ctrl</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>Selection grew from 0 or 1 node to 2+</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>Explore</x:v>
+      </x:c>
+      <x:c r="E16" t="str">
+        <x:v>Retain</x:v>
+      </x:c>
+      <x:c r="F16" t="str">
+        <x:v>Clear</x:v>
+      </x:c>
+      <x:c r="G16" t="str">
+        <x:v>Preserve current framing</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d6d506f44244e33"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3384864ddc43436b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4819,7 +4842,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="85" t="str">
-        <x:v>Focus keeps the constellation legible, grays the local neighborhood, and removes everything else.</x:v>
+        <x:v>Focus highlights its local neighborhood and selected constellation, and removes everything else.</x:v>
       </x:c>
       <x:c r="B3" s="85"/>
       <x:c r="C3" s="85"/>
@@ -4864,13 +4887,13 @@
         <x:v>Focused node, selected</x:v>
       </x:c>
       <x:c r="B7" s="105" t="str">
-        <x:v>Rendered and lit</x:v>
+        <x:v>Rendered and highlighted</x:v>
       </x:c>
       <x:c r="C7" s="105" t="str">
         <x:v>Normal local label policy</x:v>
       </x:c>
       <x:c r="D7" s="105" t="str">
-        <x:v>Focus-neighbor links remain</x:v>
+        <x:v>Focus-neighbor links highlighted</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
@@ -4878,13 +4901,13 @@
         <x:v>Focused node, unselected</x:v>
       </x:c>
       <x:c r="B8" s="101" t="str">
-        <x:v>Rendered gray; no focus-specific selection color</x:v>
+        <x:v>Rendered and highlighted</x:v>
       </x:c>
       <x:c r="C8" s="101" t="str">
         <x:v>Normal local label policy</x:v>
       </x:c>
       <x:c r="D8" s="101" t="str">
-        <x:v>Focus-neighbor links gray unless selected-selected</x:v>
+        <x:v>Focus-neighbor links highlighted</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
@@ -4892,13 +4915,13 @@
         <x:v>Immediate neighbor, unselected</x:v>
       </x:c>
       <x:c r="B9" s="105" t="str">
-        <x:v>Rendered gray</x:v>
+        <x:v>Rendered and highlighted</x:v>
       </x:c>
       <x:c r="C9" s="105" t="str">
         <x:v>Normal local label policy</x:v>
       </x:c>
       <x:c r="D9" s="105" t="str">
-        <x:v>Link to focused node rendered gray</x:v>
+        <x:v>Link to focused node highlighted</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
@@ -4932,7 +4955,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83262f55c73443cb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R948082b1a2fc4200"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5253,7 +5276,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8dddb693191e419f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc2c730c512d455b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5632,10 +5655,10 @@
         <x:v>Same</x:v>
       </x:c>
       <x:c r="E18" s="101" t="str">
-        <x:v>Focus remains valid while selection non-empty</x:v>
+        <x:v>Focus retained while held; a new multi-node constellation enters Explore on release</x:v>
       </x:c>
       <x:c r="F18" s="101" t="str">
-        <x:v>No camera change while held</x:v>
+        <x:v>No camera change while held or on release</x:v>
       </x:c>
       <x:c r="G18" s="103" t="str">
         <x:v>Implemented</x:v>
@@ -5883,7 +5906,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7be154686bda4921"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb6fb8f4964c7492b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6150,7 +6173,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reded927e8614411e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9120c1510cae48ae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6312,16 +6335,16 @@
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
       <x:c r="A11" s="105" t="str">
-        <x:v>Release Ctrl after initial selection</x:v>
+        <x:v>Release Ctrl after zero/one-node selection</x:v>
       </x:c>
       <x:c r="B11" s="105" t="str">
-        <x:v>Center + Fit result</x:v>
+        <x:v>One node: Center + Fit Focus; multiple nodes: preserve framing</x:v>
       </x:c>
       <x:c r="C11" s="105" t="str">
         <x:v>Same</x:v>
       </x:c>
       <x:c r="D11" s="105" t="str">
-        <x:v>Use resulting state target</x:v>
+        <x:v>One node: Focus; multiple nodes: Explore</x:v>
       </x:c>
       <x:c r="E11" s="103" t="str">
         <x:v>Implemented</x:v>
@@ -6331,7 +6354,7 @@
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
       <x:c r="A12" s="101" t="str">
-        <x:v>Release Ctrl after existing-selection edits</x:v>
+        <x:v>Release Ctrl after established multi-selection edits</x:v>
       </x:c>
       <x:c r="B12" s="101" t="str">
         <x:v>No camera change</x:v>
@@ -6340,7 +6363,7 @@
         <x:v>Same</x:v>
       </x:c>
       <x:c r="D12" s="101" t="str">
-        <x:v>Retain changes and Focus</x:v>
+        <x:v>Retain changes and current Explore / Focus state</x:v>
       </x:c>
       <x:c r="E12" s="103" t="str">
         <x:v>Implemented</x:v>
@@ -6471,7 +6494,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05cc6e7d69be4db8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf6c4d28e3494f41"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6994,7 +7017,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb41ee173fbfa42d4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6512245eec074c8e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7246,7 +7269,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b2682192f434969"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6b4c0392e2544ef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7451,7 +7474,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f5c1c785de347fd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6b24e672e984aef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7737,7 +7760,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b8b60d49eaf4daf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R334f2c0b86e240f8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(graph-engine): refine interaction and motion semantics
</commit_message>
<xml_diff>
--- a/docs/graph-plus-ui-interaction-matrix.xlsx
+++ b/docs/graph-plus-ui-interaction-matrix.xlsx
@@ -2,23 +2,25 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Index" sheetId="1" r:id="R8cc5b61620864eea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Definitions" sheetId="2" r:id="Rb85033a6d181416e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Desktop Pointer" sheetId="3" r:id="R07cd7d55ef7a476e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Desktop Trackpad" sheetId="4" r:id="R3c19a54f1dbc4108"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keyboard" sheetId="5" r:id="R7ce3b2f2a906428c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mobile Touch" sheetId="6" r:id="Re7ac96b293ed4fca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mobile Two-Finger" sheetId="7" r:id="Rd2463b5dcd0d4988"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stylus" sheetId="8" r:id="Ra9e0cce182d5419d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Centering" sheetId="9" r:id="R818365b1f8fc4837"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Node Context Menu" sheetId="10" r:id="Reefb1635313048b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Settings UI" sheetId="11" r:id="R70af8ee51a244a2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Settings Controls" sheetId="12" r:id="R13f8e582173049af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Note Preview" sheetId="13" r:id="R7553edd5b3774a5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Decisions" sheetId="14" r:id="R8cf13a0cd7f84ee0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Policies" sheetId="15" r:id="Rc470dda50a7945f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Transitions" sheetId="16" r:id="R675a458e26314751"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Focus Rendering" sheetId="17" r:id="R2f741878f89b4729"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Index" sheetId="1" r:id="R4de34eae769148ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Definitions" sheetId="2" r:id="R95d64a0f88ab4874"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Desktop Pointer" sheetId="3" r:id="R28e0af42b68740a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Desktop Trackpad" sheetId="4" r:id="R58a78be2e03a4131"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keyboard" sheetId="5" r:id="R4ab25627cc3a4f44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mobile Touch" sheetId="6" r:id="Ra45ef81b19674e9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mobile Two-Finger" sheetId="7" r:id="R503910370f1d472b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stylus" sheetId="8" r:id="Rfd69a5401359485f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Centering" sheetId="9" r:id="R96aa6f1ddefa4c73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Node Context Menu" sheetId="10" r:id="R556779a393134775"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Settings UI" sheetId="11" r:id="R623197351b5d468f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Settings Controls" sheetId="12" r:id="Rd98b111ee0074696"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Note Preview" sheetId="13" r:id="R5dbeb924a503420b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Decisions" sheetId="14" r:id="R9fb8c82e3ad94898"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Policies" sheetId="15" r:id="Rd3483e7b5b1c48f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Transitions" sheetId="16" r:id="R3516ce5ec02d4d81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Focus Rendering" sheetId="17" r:id="R2b8118181aba4f1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Explore Rendering" sheetId="18" r:id="R097d3123964b4cdd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persistence" sheetId="19" r:id="R71ce9a51b74e427f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -29,7 +31,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="14">
+  <x:fonts count="19">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -108,8 +110,37 @@
       <x:color rgb="FF8A5B00"/>
       <x:name val="Aptos"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF334155"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="16"/>
+      <x:color rgb="FF243B53"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF64748B"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF334155"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF334155"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="44">
+  <x:fills count="50">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -326,8 +357,38 @@
         <x:fgColor rgb="FFFFF3D3"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF243B53"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF243B53"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4F7FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3D3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE5F3EA"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="7">
+  <x:borders count="8">
     <x:border/>
     <x:border>
       <x:bottom style="thin">
@@ -383,11 +444,25 @@
         <x:color rgb="FFCFD8E3"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD5DEE8"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD5DEE8"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD5DEE8"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD5DEE8"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="108">
+  <x:cellXfs count="138">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -694,6 +769,82 @@
     <x:xf numFmtId="0" fontId="13" fillId="43" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="46" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="46" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="46" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="47" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="47" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="47" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="47" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="47" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="48" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="48" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="49" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="49" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -2662,7 +2813,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="ReviewIndexContract" displayName="ReviewIndexContract" ref="A5:E21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="ReviewIndexContract" displayName="ReviewIndexContract" ref="A5:E23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Worksheet"/>
     <x:tableColumn id="2" name="Scope"/>
@@ -2688,7 +2839,7 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="27" name="OpenDecisionsContract" displayName="OpenDecisionsContract" ref="A5:C8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="27" name="OpenDecisionsContract" displayName="OpenDecisionsContract" ref="A5:C10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="Topic"/>
     <x:tableColumn id="2" name="Current decision"/>
@@ -3338,7 +3489,7 @@
         <x:v>Explicitly deferred follow-up design</x:v>
       </x:c>
       <x:c r="C21" s="105" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D21" s="103" t="str">
         <x:v>Approved</x:v>
@@ -3346,6 +3497,36 @@
       <x:c r="E21" s="105" t="str">
         <x:v>No contract inconsistency remains</x:v>
       </x:c>
+    </x:row>
+    <x:row r="22" ht="36" customHeight="1">
+      <x:c r="A22" s="128" t="str">
+        <x:v>Explore Rendering</x:v>
+      </x:c>
+      <x:c r="B22" s="128" t="str">
+        <x:v>Constellation emphasis, context dimming, and hover inspection</x:v>
+      </x:c>
+      <x:c r="C22" s="128" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D22" s="137" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+      <x:c r="E22" s="128"/>
+    </x:row>
+    <x:row r="23" ht="36" customHeight="1">
+      <x:c r="A23" s="133" t="str">
+        <x:v>Persistence</x:v>
+      </x:c>
+      <x:c r="B23" s="133" t="str">
+        <x:v>Saved-view restoration and initial framing</x:v>
+      </x:c>
+      <x:c r="C23" s="133" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D23" s="137" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+      <x:c r="E23" s="133"/>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="D6:D18">
@@ -3360,7 +3541,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfea1b0e8c1b145f4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98d7520c0c874cd2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3519,7 +3700,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb502d435a5244c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rca1e439087d24176"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4242,17 +4423,29 @@
       <x:c r="D8"/>
       <x:c r="E8"/>
     </x:row>
-    <x:row r="9" ht="43" customHeight="1">
-      <x:c r="A9"/>
-      <x:c r="B9"/>
-      <x:c r="C9"/>
+    <x:row r="9" ht="52" customHeight="1">
+      <x:c r="A9" s="128" t="str">
+        <x:v>Anima hover resistance</x:v>
+      </x:c>
+      <x:c r="B9" s="128" t="str">
+        <x:v>Require dwell and movement resistance before a dim Explore node becomes transiently lit; immediate hover remains the interim behavior.</x:v>
+      </x:c>
+      <x:c r="C9" s="135" t="str">
+        <x:v>Deferred</x:v>
+      </x:c>
       <x:c r="D9"/>
       <x:c r="E9"/>
     </x:row>
-    <x:row r="10" ht="43" customHeight="1">
-      <x:c r="A10"/>
-      <x:c r="B10"/>
-      <x:c r="C10"/>
+    <x:row r="10" ht="52" customHeight="1">
+      <x:c r="A10" s="133" t="str">
+        <x:v>Shading and color language</x:v>
+      </x:c>
+      <x:c r="B10" s="133" t="str">
+        <x:v>Develop a shared Anima shading and color language; current Explore baseline is 24% opacity with 80% desaturation.</x:v>
+      </x:c>
+      <x:c r="C10" s="135" t="str">
+        <x:v>Deferred</x:v>
+      </x:c>
       <x:c r="D10"/>
       <x:c r="E10"/>
     </x:row>
@@ -4320,7 +4513,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58a39c9bc09b4f29"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c98c68a33e64c36"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4451,7 +4644,7 @@
         <x:v>Pan</x:v>
       </x:c>
       <x:c r="H7" s="105" t="str">
-        <x:v>Rotate</x:v>
+        <x:v>Pan</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
@@ -4483,7 +4676,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b5965d5a41445ae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f0245106f964a16"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4569,16 +4762,16 @@
         <x:v>Any visible node</x:v>
       </x:c>
       <x:c r="D6" s="101" t="str">
-        <x:v>Focus</x:v>
+        <x:v>Explore</x:v>
       </x:c>
       <x:c r="E6" s="101" t="str">
         <x:v>Select node</x:v>
       </x:c>
       <x:c r="F6" s="101" t="str">
-        <x:v>Focus clicked node</x:v>
+        <x:v>Clear</x:v>
       </x:c>
       <x:c r="G6" s="101" t="str">
-        <x:v>Center node; fit immediate neighbors</x:v>
+        <x:v>No camera change</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
@@ -4615,16 +4808,16 @@
         <x:v>Stationary</x:v>
       </x:c>
       <x:c r="D8" s="101" t="str">
-        <x:v>Focus</x:v>
+        <x:v>Explore or Overview</x:v>
       </x:c>
       <x:c r="E8" s="101" t="str">
-        <x:v>No change</x:v>
+        <x:v>Remove clicked node</x:v>
       </x:c>
       <x:c r="F8" s="101" t="str">
-        <x:v>Focus clicked node</x:v>
+        <x:v>Clear</x:v>
       </x:c>
       <x:c r="G8" s="101" t="str">
-        <x:v>Center node; fit immediate neighbors</x:v>
+        <x:v>No camera change</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
@@ -4647,7 +4840,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G9" s="105" t="str">
-        <x:v>Center + Fit graph</x:v>
+        <x:v>No camera change</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
@@ -4655,22 +4848,22 @@
         <x:v>Focus</x:v>
       </x:c>
       <x:c r="B10" s="101" t="str">
-        <x:v>Click different visible node</x:v>
+        <x:v>Click unselected node</x:v>
       </x:c>
       <x:c r="C10" s="101" t="str">
         <x:v>Stationary</x:v>
       </x:c>
       <x:c r="D10" s="101" t="str">
-        <x:v>Focus</x:v>
+        <x:v>Explore</x:v>
       </x:c>
       <x:c r="E10" s="101" t="str">
-        <x:v>No change</x:v>
+        <x:v>Add node + shortest-path bridge</x:v>
       </x:c>
       <x:c r="F10" s="101" t="str">
-        <x:v>Hop to clicked node</x:v>
+        <x:v>Clear</x:v>
       </x:c>
       <x:c r="G10" s="101" t="str">
-        <x:v>Center node; fit immediate neighbors</x:v>
+        <x:v>No camera change</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
@@ -4678,22 +4871,22 @@
         <x:v>Focus</x:v>
       </x:c>
       <x:c r="B11" s="105" t="str">
-        <x:v>Single click focused node</x:v>
+        <x:v>Click selected node</x:v>
       </x:c>
       <x:c r="C11" s="105" t="str">
-        <x:v>After double-click arbitration</x:v>
+        <x:v>Stationary after double-click arbitration</x:v>
       </x:c>
       <x:c r="D11" s="105" t="str">
-        <x:v>Focus or Overview</x:v>
+        <x:v>Explore or Overview</x:v>
       </x:c>
       <x:c r="E11" s="105" t="str">
-        <x:v>Toggle focused node</x:v>
+        <x:v>Remove clicked node</x:v>
       </x:c>
       <x:c r="F11" s="105" t="str">
-        <x:v>Retain unless selection becomes empty</x:v>
+        <x:v>Clear</x:v>
       </x:c>
       <x:c r="G11" s="105" t="str">
-        <x:v>Fit graph only if selection becomes empty</x:v>
+        <x:v>No camera change</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
@@ -4716,7 +4909,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G12" s="101" t="str">
-        <x:v>Center + Fit selection</x:v>
+        <x:v>No camera change</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
@@ -4739,7 +4932,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G13" s="105" t="str">
-        <x:v>Center + Fit graph</x:v>
+        <x:v>No camera change</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
@@ -4747,16 +4940,16 @@
         <x:v>Any</x:v>
       </x:c>
       <x:c r="B14" s="101" t="str">
-        <x:v>Double-click / tap focused node</x:v>
+        <x:v>Double-click / tap node</x:v>
       </x:c>
       <x:c r="C14" s="101" t="str">
-        <x:v>Focused before first activation</x:v>
+        <x:v>Same node twice without drag</x:v>
       </x:c>
       <x:c r="D14" s="101" t="str">
         <x:v>Same</x:v>
       </x:c>
       <x:c r="E14" s="101" t="str">
-        <x:v>No change</x:v>
+        <x:v>Leave node selected</x:v>
       </x:c>
       <x:c r="F14" s="101" t="str">
         <x:v>No change</x:v>
@@ -4790,31 +4983,31 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="str">
-        <x:v>Focus</x:v>
+        <x:v>Any</x:v>
       </x:c>
       <x:c r="B16" t="str">
         <x:v>Release Ctrl</x:v>
       </x:c>
       <x:c r="C16" t="str">
-        <x:v>Selection grew from 0 or 1 node to 2+</x:v>
+        <x:v>Any selection</x:v>
       </x:c>
       <x:c r="D16" t="str">
-        <x:v>Explore</x:v>
+        <x:v>Same</x:v>
       </x:c>
       <x:c r="E16" t="str">
         <x:v>Retain</x:v>
       </x:c>
       <x:c r="F16" t="str">
-        <x:v>Clear</x:v>
+        <x:v>No change</x:v>
       </x:c>
       <x:c r="G16" t="str">
-        <x:v>Preserve current framing</x:v>
+        <x:v>No camera change</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3384864ddc43436b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra939a9afc2274ef4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4955,8 +5148,263 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R948082b1a2fc4200"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5833709323ba46ae"/>
   </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="21.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="31.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="31.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="31.670000076293945" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="2">
+      <x:c r="A2" s="110" t="str">
+        <x:v>Explore / Constellation rendering</x:v>
+      </x:c>
+      <x:c r="B2" s="109"/>
+      <x:c r="C2" s="109"/>
+      <x:c r="D2" s="109"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="112" t="str">
+        <x:v>Selected structure remains durable; dim graph context stays inspectable without changing selection.</x:v>
+      </x:c>
+      <x:c r="B3" s="109"/>
+      <x:c r="C3" s="109"/>
+      <x:c r="D3" s="109"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="109"/>
+      <x:c r="B4" s="109"/>
+      <x:c r="C4" s="109"/>
+      <x:c r="D4" s="109"/>
+    </x:row>
+    <x:row r="5" ht="28" customHeight="1">
+      <x:c r="A5" s="123" t="str">
+        <x:v>Element</x:v>
+      </x:c>
+      <x:c r="B5" s="123" t="str">
+        <x:v>Node presentation</x:v>
+      </x:c>
+      <x:c r="C5" s="123" t="str">
+        <x:v>Label presentation</x:v>
+      </x:c>
+      <x:c r="D5" s="123" t="str">
+        <x:v>Link presentation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="42" customHeight="1">
+      <x:c r="A6" s="118" t="str">
+        <x:v>Selected constellation node</x:v>
+      </x:c>
+      <x:c r="B6" s="118" t="str">
+        <x:v>Full opacity; accent highlight</x:v>
+      </x:c>
+      <x:c r="C6" s="118" t="str">
+        <x:v>Selected emphasis</x:v>
+      </x:c>
+      <x:c r="D6" s="118" t="str">
+        <x:v>Selected-to-selected links lit</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="42" customHeight="1">
+      <x:c r="A7" s="118" t="str">
+        <x:v>Unselected context node</x:v>
+      </x:c>
+      <x:c r="B7" s="118" t="str">
+        <x:v>24% opacity; ordinary theme color with 80% desaturation</x:v>
+      </x:c>
+      <x:c r="C7" s="118" t="str">
+        <x:v>Normal adaptive policy; dim context</x:v>
+      </x:c>
+      <x:c r="D7" s="118" t="str">
+        <x:v>Incident links remain dim</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="42" customHeight="1">
+      <x:c r="A8" s="118" t="str">
+        <x:v>Hovered context node</x:v>
+      </x:c>
+      <x:c r="B8" s="118" t="str">
+        <x:v>Transient full highlight; no selection change</x:v>
+      </x:c>
+      <x:c r="C8" s="118" t="str">
+        <x:v>Force hovered label visible</x:v>
+      </x:c>
+      <x:c r="D8" s="118" t="str">
+        <x:v>Neighbors, path, and incident links remain dim</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="42" customHeight="1">
+      <x:c r="A9" s="118" t="str">
+        <x:v>Previewed or Option-revealed context</x:v>
+      </x:c>
+      <x:c r="B9" s="118" t="str">
+        <x:v>Remain dim outside the constellation</x:v>
+      </x:c>
+      <x:c r="C9" s="118" t="str">
+        <x:v>No automatic promotion</x:v>
+      </x:c>
+      <x:c r="D9" s="118" t="str">
+        <x:v>Remain dim</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="42" customHeight="1">
+      <x:c r="A10" s="118" t="str">
+        <x:v>Hover resistance</x:v>
+      </x:c>
+      <x:c r="B10" s="118" t="str">
+        <x:v>Immediate interim behavior; dwell and movement resistance deferred to shared Anima animation kit</x:v>
+      </x:c>
+      <x:c r="C10" s="118" t="str">
+        <x:v>No state change</x:v>
+      </x:c>
+      <x:c r="D10" s="118" t="str">
+        <x:v>No state change</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A2:D2"/>
+    <x:mergeCell ref="A3:D3"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22.219999313354492" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="30" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="30" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="11.670000076293945" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="2">
+      <x:c r="A2" s="110" t="str">
+        <x:v>Saved view restoration</x:v>
+      </x:c>
+      <x:c r="B2" s="109"/>
+      <x:c r="C2" s="109"/>
+      <x:c r="D2" s="109"/>
+      <x:c r="E2" s="109"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="112" t="str">
+        <x:v>Loading a graph should return to its last compatible state without an automatic camera move.</x:v>
+      </x:c>
+      <x:c r="B3" s="109"/>
+      <x:c r="C3" s="109"/>
+      <x:c r="D3" s="109"/>
+      <x:c r="E3" s="109"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="109"/>
+      <x:c r="B4" s="109"/>
+      <x:c r="C4" s="109"/>
+      <x:c r="D4" s="109"/>
+      <x:c r="E4" s="109"/>
+    </x:row>
+    <x:row r="5" ht="28" customHeight="1">
+      <x:c r="A5" s="123" t="str">
+        <x:v>Situation</x:v>
+      </x:c>
+      <x:c r="B5" s="123" t="str">
+        <x:v>Restored state</x:v>
+      </x:c>
+      <x:c r="C5" s="123" t="str">
+        <x:v>Camera behavior</x:v>
+      </x:c>
+      <x:c r="D5" s="123" t="str">
+        <x:v>Fallback</x:v>
+      </x:c>
+      <x:c r="E5" s="123" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="42" customHeight="1">
+      <x:c r="A6" s="118" t="str">
+        <x:v>Compatible saved Graph+ view</x:v>
+      </x:c>
+      <x:c r="B6" s="118" t="str">
+        <x:v>Positions, pins, selection, Focus, filters, Form/module state</x:v>
+      </x:c>
+      <x:c r="C6" s="118" t="str">
+        <x:v>Restore saved framing; do not center or fit</x:v>
+      </x:c>
+      <x:c r="D6" s="118" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E6" s="118" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="42" customHeight="1">
+      <x:c r="A7" s="118" t="str">
+        <x:v>Saved graph reconciles with vault</x:v>
+      </x:c>
+      <x:c r="B7" s="118" t="str">
+        <x:v>Reconcile by stable IDs</x:v>
+      </x:c>
+      <x:c r="C7" s="118" t="str">
+        <x:v>Preserve restored framing</x:v>
+      </x:c>
+      <x:c r="D7" s="118" t="str">
+        <x:v>Drop only incompatible IDs or state</x:v>
+      </x:c>
+      <x:c r="E7" s="118" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="42" customHeight="1">
+      <x:c r="A8" s="118" t="str">
+        <x:v>No compatible saved view</x:v>
+      </x:c>
+      <x:c r="B8" s="118" t="str">
+        <x:v>Fresh Overview</x:v>
+      </x:c>
+      <x:c r="C8" s="118" t="str">
+        <x:v>Initial whole-graph fit</x:v>
+      </x:c>
+      <x:c r="D8" s="118" t="str">
+        <x:v>Generate finite positions</x:v>
+      </x:c>
+      <x:c r="E8" s="118" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="42" customHeight="1">
+      <x:c r="A9" s="118" t="str">
+        <x:v>Explicit layout reset</x:v>
+      </x:c>
+      <x:c r="B9" s="118" t="str">
+        <x:v>Discard saved layout and interaction state</x:v>
+      </x:c>
+      <x:c r="C9" s="118" t="str">
+        <x:v>Explicit whole-graph fit is allowed</x:v>
+      </x:c>
+      <x:c r="D9" s="118" t="str">
+        <x:v>Create a fresh checkpoint</x:v>
+      </x:c>
+      <x:c r="E9" s="118" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A2:E2"/>
+    <x:mergeCell ref="A3:E3"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
 
@@ -5129,7 +5577,7 @@
         <x:v>Changes framing without changing selection.</x:v>
       </x:c>
       <x:c r="D12" s="101" t="str">
-        <x:v>Normal in Overview and 2D Explore</x:v>
+        <x:v>Normal in Overview and Explore</x:v>
       </x:c>
       <x:c r="E12" s="103" t="str">
         <x:v>Implemented</x:v>
@@ -5163,7 +5611,7 @@
         <x:v>Changes angle without fitting or recentering.</x:v>
       </x:c>
       <x:c r="D14" s="101" t="str">
-        <x:v>Default 3D Explore and Focus navigation</x:v>
+        <x:v>Secondary drag in 3D Explore; primary navigation in 3D Focus</x:v>
       </x:c>
       <x:c r="E14" s="103" t="str">
         <x:v>Implemented</x:v>
@@ -5276,7 +5724,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc2c730c512d455b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra30394f0d7f54ffa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5358,16 +5806,16 @@
         <x:v>Hover</x:v>
       </x:c>
       <x:c r="B6" s="101" t="str">
-        <x:v>Node / any state</x:v>
+        <x:v>Node / Overview or Explore</x:v>
       </x:c>
       <x:c r="C6" s="101" t="str">
-        <x:v>Highlight node</x:v>
+        <x:v>Highlight hovered node only</x:v>
       </x:c>
       <x:c r="D6" s="101" t="str">
-        <x:v>Highlight node</x:v>
+        <x:v>Highlight hovered node only</x:v>
       </x:c>
       <x:c r="E6" s="101" t="str">
-        <x:v>No state change</x:v>
+        <x:v>No selection change</x:v>
       </x:c>
       <x:c r="F6" s="101" t="str">
         <x:v>Transient only</x:v>
@@ -5442,7 +5890,7 @@
         <x:v>Enter Overview</x:v>
       </x:c>
       <x:c r="F9" s="105" t="str">
-        <x:v>Center + Fit graph</x:v>
+        <x:v>No camera change</x:v>
       </x:c>
       <x:c r="G9" s="103" t="str">
         <x:v>Implemented</x:v>
@@ -5466,7 +5914,7 @@
         <x:v>Enter Explore</x:v>
       </x:c>
       <x:c r="F10" s="101" t="str">
-        <x:v>Center + Fit selection</x:v>
+        <x:v>No camera change</x:v>
       </x:c>
       <x:c r="G10" s="103" t="str">
         <x:v>Implemented</x:v>
@@ -5490,7 +5938,7 @@
         <x:v>Enter Overview</x:v>
       </x:c>
       <x:c r="F11" s="105" t="str">
-        <x:v>Center + Fit graph</x:v>
+        <x:v>No camera change</x:v>
       </x:c>
       <x:c r="G11" s="103" t="str">
         <x:v>Implemented</x:v>
@@ -5505,16 +5953,16 @@
         <x:v>Node / Overview</x:v>
       </x:c>
       <x:c r="C12" s="101" t="str">
-        <x:v>Select + Focus</x:v>
+        <x:v>Select; enter Explore</x:v>
       </x:c>
       <x:c r="D12" s="101" t="str">
         <x:v>Same</x:v>
       </x:c>
       <x:c r="E12" s="101" t="str">
-        <x:v>Enter Focus</x:v>
+        <x:v>Select node; clear Focus</x:v>
       </x:c>
       <x:c r="F12" s="101" t="str">
-        <x:v>Center node; fit immediate neighbors</x:v>
+        <x:v>No camera change</x:v>
       </x:c>
       <x:c r="G12" s="103" t="str">
         <x:v>Implemented</x:v>
@@ -5553,16 +6001,16 @@
         <x:v>Selected node / Explore</x:v>
       </x:c>
       <x:c r="C14" s="101" t="str">
-        <x:v>Enter Focus</x:v>
+        <x:v>Remove node</x:v>
       </x:c>
       <x:c r="D14" s="101" t="str">
         <x:v>Same</x:v>
       </x:c>
       <x:c r="E14" s="101" t="str">
-        <x:v>Selection unchanged</x:v>
+        <x:v>Remain Explore, or Overview if empty</x:v>
       </x:c>
       <x:c r="F14" s="101" t="str">
-        <x:v>Center node; fit immediate neighbors</x:v>
+        <x:v>No camera change</x:v>
       </x:c>
       <x:c r="G14" s="103" t="str">
         <x:v>Implemented</x:v>
@@ -5574,19 +6022,19 @@
         <x:v>Primary click</x:v>
       </x:c>
       <x:c r="B15" s="105" t="str">
-        <x:v>Different local node / Focus</x:v>
+        <x:v>Unselected node / Focus</x:v>
       </x:c>
       <x:c r="C15" s="105" t="str">
-        <x:v>Hop Focus</x:v>
+        <x:v>Add node + path bridge; exit Focus</x:v>
       </x:c>
       <x:c r="D15" s="105" t="str">
         <x:v>Same</x:v>
       </x:c>
       <x:c r="E15" s="105" t="str">
-        <x:v>Selection unchanged</x:v>
+        <x:v>Enter Explore</x:v>
       </x:c>
       <x:c r="F15" s="105" t="str">
-        <x:v>Center node; fit immediate neighbors</x:v>
+        <x:v>No camera change</x:v>
       </x:c>
       <x:c r="G15" s="103" t="str">
         <x:v>Implemented</x:v>
@@ -5598,19 +6046,19 @@
         <x:v>Primary click</x:v>
       </x:c>
       <x:c r="B16" s="101" t="str">
-        <x:v>Focused node / Focus</x:v>
+        <x:v>Selected node / Focus</x:v>
       </x:c>
       <x:c r="C16" s="101" t="str">
-        <x:v>Toggle membership after double-click delay</x:v>
+        <x:v>Remove node; exit Focus</x:v>
       </x:c>
       <x:c r="D16" s="101" t="str">
         <x:v>Same</x:v>
       </x:c>
       <x:c r="E16" s="101" t="str">
-        <x:v>Focus independent of membership</x:v>
+        <x:v>Enter Explore, or Overview if empty</x:v>
       </x:c>
       <x:c r="F16" s="101" t="str">
-        <x:v>Graph fit only if selection empties</x:v>
+        <x:v>No camera change</x:v>
       </x:c>
       <x:c r="G16" s="103" t="str">
         <x:v>Implemented</x:v>
@@ -5622,7 +6070,7 @@
         <x:v>Double click</x:v>
       </x:c>
       <x:c r="B17" s="105" t="str">
-        <x:v>Already-focused node</x:v>
+        <x:v>Node</x:v>
       </x:c>
       <x:c r="C17" s="105" t="str">
         <x:v>Primary node action</x:v>
@@ -5631,7 +6079,7 @@
         <x:v>Same</x:v>
       </x:c>
       <x:c r="E17" s="105" t="str">
-        <x:v>No state change</x:v>
+        <x:v>Leave node selected</x:v>
       </x:c>
       <x:c r="F17" s="105" t="str">
         <x:v>No camera change</x:v>
@@ -5649,16 +6097,16 @@
         <x:v>Node</x:v>
       </x:c>
       <x:c r="C18" s="101" t="str">
-        <x:v>Add / remove selection</x:v>
+        <x:v>Same as primary click</x:v>
       </x:c>
       <x:c r="D18" s="101" t="str">
         <x:v>Same</x:v>
       </x:c>
       <x:c r="E18" s="101" t="str">
-        <x:v>Focus retained while held; a new multi-node constellation enters Explore on release</x:v>
+        <x:v>Toggle constellation membership; clear Focus</x:v>
       </x:c>
       <x:c r="F18" s="101" t="str">
-        <x:v>No camera change while held or on release</x:v>
+        <x:v>No camera change</x:v>
       </x:c>
       <x:c r="G18" s="103" t="str">
         <x:v>Implemented</x:v>
@@ -5700,13 +6148,13 @@
         <x:v>Pan</x:v>
       </x:c>
       <x:c r="D20" s="101" t="str">
-        <x:v>Rotate</x:v>
+        <x:v>Pan</x:v>
       </x:c>
       <x:c r="E20" s="101" t="str">
         <x:v>Retain selection</x:v>
       </x:c>
       <x:c r="F20" s="101" t="str">
-        <x:v>State-owned navigation</x:v>
+        <x:v>Translate camera</x:v>
       </x:c>
       <x:c r="G20" s="103" t="str">
         <x:v>Implemented</x:v>
@@ -5906,7 +6354,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb6fb8f4964c7492b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd0764b7ff38d4250"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6173,7 +6621,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9120c1510cae48ae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1421ca1168ba4d3c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6319,13 +6767,13 @@
         <x:v>Hold Ctrl + node clicks</x:v>
       </x:c>
       <x:c r="B10" s="101" t="str">
-        <x:v>Edit selection</x:v>
+        <x:v>Same selection toggle as primary click</x:v>
       </x:c>
       <x:c r="C10" s="101" t="str">
         <x:v>Same</x:v>
       </x:c>
       <x:c r="D10" s="101" t="str">
-        <x:v>No camera change during edits</x:v>
+        <x:v>Additions include shortest path; no camera change</x:v>
       </x:c>
       <x:c r="E10" s="103" t="str">
         <x:v>Implemented</x:v>
@@ -6335,16 +6783,16 @@
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
       <x:c r="A11" s="105" t="str">
-        <x:v>Release Ctrl after zero/one-node selection</x:v>
+        <x:v>Release Ctrl</x:v>
       </x:c>
       <x:c r="B11" s="105" t="str">
-        <x:v>One node: Center + Fit Focus; multiple nodes: preserve framing</x:v>
+        <x:v>No change</x:v>
       </x:c>
       <x:c r="C11" s="105" t="str">
         <x:v>Same</x:v>
       </x:c>
       <x:c r="D11" s="105" t="str">
-        <x:v>One node: Focus; multiple nodes: Explore</x:v>
+        <x:v>Preserve selection, state, and framing</x:v>
       </x:c>
       <x:c r="E11" s="103" t="str">
         <x:v>Implemented</x:v>
@@ -6354,7 +6802,7 @@
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
       <x:c r="A12" s="101" t="str">
-        <x:v>Release Ctrl after established multi-selection edits</x:v>
+        <x:v>Release Ctrl after selection edits</x:v>
       </x:c>
       <x:c r="B12" s="101" t="str">
         <x:v>No camera change</x:v>
@@ -6363,7 +6811,7 @@
         <x:v>Same</x:v>
       </x:c>
       <x:c r="D12" s="101" t="str">
-        <x:v>Retain changes and current Explore / Focus state</x:v>
+        <x:v>Preserve selection, state, and framing</x:v>
       </x:c>
       <x:c r="E12" s="103" t="str">
         <x:v>Implemented</x:v>
@@ -6376,7 +6824,7 @@
         <x:v>Hold Option</x:v>
       </x:c>
       <x:c r="B13" s="105" t="str">
-        <x:v>Reveal neighbors + connecting links</x:v>
+        <x:v>Preserve constellation-only highlighting</x:v>
       </x:c>
       <x:c r="C13" s="105" t="str">
         <x:v>Same</x:v>
@@ -6494,7 +6942,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf6c4d28e3494f41"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16d4aa6bb3ad4e1c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6612,7 +7060,7 @@
         <x:v>Enter Overview</x:v>
       </x:c>
       <x:c r="F7" s="105" t="str">
-        <x:v>Center + Fit graph</x:v>
+        <x:v>No camera change</x:v>
       </x:c>
       <x:c r="G7" s="103" t="str">
         <x:v>Implemented</x:v>
@@ -6636,7 +7084,7 @@
         <x:v>Enter Explore</x:v>
       </x:c>
       <x:c r="F8" s="101" t="str">
-        <x:v>Center + Fit selection</x:v>
+        <x:v>No camera change</x:v>
       </x:c>
       <x:c r="G8" s="103" t="str">
         <x:v>Implemented</x:v>
@@ -6660,7 +7108,7 @@
         <x:v>Enter Overview</x:v>
       </x:c>
       <x:c r="F9" s="105" t="str">
-        <x:v>Center + Fit graph</x:v>
+        <x:v>No camera change</x:v>
       </x:c>
       <x:c r="G9" s="103" t="str">
         <x:v>Implemented</x:v>
@@ -6675,16 +7123,16 @@
         <x:v>Node / Overview</x:v>
       </x:c>
       <x:c r="C10" s="101" t="str">
-        <x:v>Select + Focus on release</x:v>
+        <x:v>Select on release; enter Explore</x:v>
       </x:c>
       <x:c r="D10" s="101" t="str">
         <x:v>Same</x:v>
       </x:c>
       <x:c r="E10" s="101" t="str">
-        <x:v>Enter Focus</x:v>
+        <x:v>Select node; clear Focus</x:v>
       </x:c>
       <x:c r="F10" s="101" t="str">
-        <x:v>Center node; fit immediate neighbors</x:v>
+        <x:v>No camera change</x:v>
       </x:c>
       <x:c r="G10" s="103" t="str">
         <x:v>Implemented</x:v>
@@ -6696,19 +7144,19 @@
         <x:v>Tap</x:v>
       </x:c>
       <x:c r="B11" s="105" t="str">
-        <x:v>Selected node / Explore</x:v>
+        <x:v>Unselected node / Explore</x:v>
       </x:c>
       <x:c r="C11" s="105" t="str">
-        <x:v>Enter Focus</x:v>
+        <x:v>Add node + path bridge</x:v>
       </x:c>
       <x:c r="D11" s="105" t="str">
         <x:v>Same</x:v>
       </x:c>
       <x:c r="E11" s="105" t="str">
-        <x:v>Selection unchanged</x:v>
+        <x:v>Remain Explore</x:v>
       </x:c>
       <x:c r="F11" s="105" t="str">
-        <x:v>Center node; fit immediate neighbors</x:v>
+        <x:v>No camera change</x:v>
       </x:c>
       <x:c r="G11" s="103" t="str">
         <x:v>Implemented</x:v>
@@ -6720,19 +7168,19 @@
         <x:v>Tap</x:v>
       </x:c>
       <x:c r="B12" s="101" t="str">
-        <x:v>Different local node / Focus</x:v>
+        <x:v>Selected node / Explore</x:v>
       </x:c>
       <x:c r="C12" s="101" t="str">
-        <x:v>Hop Focus</x:v>
+        <x:v>Remove node</x:v>
       </x:c>
       <x:c r="D12" s="101" t="str">
         <x:v>Same</x:v>
       </x:c>
       <x:c r="E12" s="101" t="str">
-        <x:v>Selection unchanged</x:v>
+        <x:v>Remain Explore, or Overview if empty</x:v>
       </x:c>
       <x:c r="F12" s="101" t="str">
-        <x:v>Center node; fit immediate neighbors</x:v>
+        <x:v>No camera change</x:v>
       </x:c>
       <x:c r="G12" s="103" t="str">
         <x:v>Implemented</x:v>
@@ -6744,19 +7192,19 @@
         <x:v>Tap</x:v>
       </x:c>
       <x:c r="B13" s="105" t="str">
-        <x:v>Focused node / Focus</x:v>
+        <x:v>Any node / Focus</x:v>
       </x:c>
       <x:c r="C13" s="105" t="str">
-        <x:v>Toggle membership after double-tap delay</x:v>
+        <x:v>Toggle membership; exit Focus</x:v>
       </x:c>
       <x:c r="D13" s="105" t="str">
         <x:v>Same</x:v>
       </x:c>
       <x:c r="E13" s="105" t="str">
-        <x:v>Focus independent of membership</x:v>
+        <x:v>Enter Explore, or Overview if empty</x:v>
       </x:c>
       <x:c r="F13" s="105" t="str">
-        <x:v>Graph fit only if selection empties</x:v>
+        <x:v>No camera change</x:v>
       </x:c>
       <x:c r="G13" s="103" t="str">
         <x:v>Implemented</x:v>
@@ -6774,7 +7222,7 @@
         <x:v>Pan</x:v>
       </x:c>
       <x:c r="D14" s="101" t="str">
-        <x:v>Rotate</x:v>
+        <x:v>Pan</x:v>
       </x:c>
       <x:c r="E14" s="101" t="str">
         <x:v>No selection or node drag</x:v>
@@ -6798,7 +7246,7 @@
         <x:v>Pan</x:v>
       </x:c>
       <x:c r="D15" s="105" t="str">
-        <x:v>Rotate</x:v>
+        <x:v>Pan</x:v>
       </x:c>
       <x:c r="E15" s="105" t="str">
         <x:v>Selection retained; no node drag</x:v>
@@ -6864,7 +7312,7 @@
         <x:v>Double tap</x:v>
       </x:c>
       <x:c r="B18" s="101" t="str">
-        <x:v>Already-focused node</x:v>
+        <x:v>Node</x:v>
       </x:c>
       <x:c r="C18" s="101" t="str">
         <x:v>Primary node action</x:v>
@@ -6873,7 +7321,7 @@
         <x:v>Same</x:v>
       </x:c>
       <x:c r="E18" s="101" t="str">
-        <x:v>No state change</x:v>
+        <x:v>Leave node selected</x:v>
       </x:c>
       <x:c r="F18" s="101" t="str">
         <x:v>No camera change</x:v>
@@ -7017,7 +7465,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6512245eec074c8e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ae5572ac29e4e03"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7269,7 +7717,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6b4c0392e2544ef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fe34b50de114424"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7474,7 +7922,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6b24e672e984aef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd222b9ad170643c8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7760,7 +8208,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R334f2c0b86e240f8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8629f7996db74e7e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>